<commit_message>
fix(web): make Excel 365 workbooks provably editable, and never re-encode legacy CSV
The save proof now allows only metadata Excel regenerates (revision pointers, the saved path, default
slicer and timeline styles, print stamps) and compares calcPr, bookViews, app.xml, note boxes and the
differential formats rules use. hucre is patched to keep base column widths, sheet code names, table
column formats, built-in number formats, styled rows past the data and calcPr, to leave unstyled cells
unstyled, and to write columns as ranges. Parts copied verbatim that name style-table ids, such as
pivots, open read-only. Typed modern functions are saved with their _xlfn prefix, sheet names with
symbols are quoted, and dynamic array sizes are bounded in the engine.

A legacy CSV is always saved in the encoding it was read in, so untouched cells come back byte for byte;
an edit its encoding cannot hold is refused instead of re-encoding the file.
</commit_message>
<xml_diff>
--- a/packages/filen-web/src/tests/fixtures/spreadsheet/excel_full.xlsx
+++ b/packages/filen-web/src/tests/fixtures/spreadsheet/excel_full.xlsx
@@ -22,7 +22,7 @@
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
-    <author>Jan</author>
+    <author>Example Author</author>
   </authors>
   <commentList>
     <comment ref="B2" authorId="0" shapeId="0" xr:uid="{11111111-2222-3333-4444-555555555555}">
@@ -35,7 +35,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>Jan:</t>
+          <t>Example Author:</t>
         </r>
         <r>
           <rPr>

</xml_diff>